<commit_message>
base pc runs 5 t/m 10
</commit_message>
<xml_diff>
--- a/dataset_agreed/saved_models/baserun/pointcloud_base_run10/epoch_10/per_file_predictions_epoch_10.xlsx
+++ b/dataset_agreed/saved_models/baserun/pointcloud_base_run10/epoch_10/per_file_predictions_epoch_10.xlsx
@@ -808,769 +808,769 @@
     <t>0,1,1,0</t>
   </si>
   <si>
-    <t>0.0586,0.9186,0.0380,0.0063</t>
-  </si>
-  <si>
-    <t>0.3622,0.2045,0.0311,0.2547</t>
-  </si>
-  <si>
-    <t>0.2277,0.7330,0.0552,0.0185</t>
-  </si>
-  <si>
-    <t>0.6637,0.1144,0.1398,0.0181</t>
-  </si>
-  <si>
-    <t>0.4029,0.3845,0.0195,0.0848</t>
-  </si>
-  <si>
-    <t>0.2880,0.5634,0.0191,0.0611</t>
-  </si>
-  <si>
-    <t>0.3288,0.6310,0.0409,0.0209</t>
-  </si>
-  <si>
-    <t>0.4336,0.4440,0.0289,0.0390</t>
-  </si>
-  <si>
-    <t>0.2315,0.7152,0.0286,0.0275</t>
-  </si>
-  <si>
-    <t>0.2698,0.6746,0.0382,0.0294</t>
-  </si>
-  <si>
-    <t>0.2787,0.5757,0.0200,0.0668</t>
-  </si>
-  <si>
-    <t>0.4524,0.4609,0.0280,0.0269</t>
-  </si>
-  <si>
-    <t>0.1319,0.7661,0.1156,0.0042</t>
-  </si>
-  <si>
-    <t>0.0447,0.8825,0.1250,0.0027</t>
-  </si>
-  <si>
-    <t>0.1249,0.5592,0.3156,0.0043</t>
-  </si>
-  <si>
-    <t>0.1618,0.2499,0.4896,0.0035</t>
-  </si>
-  <si>
-    <t>0.2914,0.5333,0.1288,0.0057</t>
-  </si>
-  <si>
-    <t>0.0141,0.9747,0.0199,0.0016</t>
-  </si>
-  <si>
-    <t>0.0205,0.9634,0.0277,0.0026</t>
-  </si>
-  <si>
-    <t>0.0175,0.9696,0.0227,0.0019</t>
-  </si>
-  <si>
-    <t>0.0194,0.9654,0.0266,0.0026</t>
-  </si>
-  <si>
-    <t>0.0051,0.9890,0.0126,0.0007</t>
-  </si>
-  <si>
-    <t>0.2490,0.4648,0.2458,0.0059</t>
-  </si>
-  <si>
-    <t>0.3218,0.1886,0.3529,0.0025</t>
-  </si>
-  <si>
-    <t>0.0858,0.0233,0.8691,0.0012</t>
-  </si>
-  <si>
-    <t>0.4159,0.0805,0.4386,0.0044</t>
-  </si>
-  <si>
-    <t>0.3555,0.0226,0.6222,0.0036</t>
-  </si>
-  <si>
-    <t>0.4582,0.0213,0.5468,0.0037</t>
-  </si>
-  <si>
-    <t>0.0241,0.0982,0.9086,0.0011</t>
-  </si>
-  <si>
-    <t>0.0115,0.9726,0.0390,0.0016</t>
-  </si>
-  <si>
-    <t>0.2609,0.6363,0.1065,0.0077</t>
-  </si>
-  <si>
-    <t>0.0000,0.2334,0.9992,0.0000</t>
-  </si>
-  <si>
-    <t>0.1123,0.6353,0.2459,0.0028</t>
-  </si>
-  <si>
-    <t>0.1911,0.7502,0.0923,0.0135</t>
-  </si>
-  <si>
-    <t>0.1321,0.7870,0.1181,0.0120</t>
-  </si>
-  <si>
-    <t>0.0662,0.9134,0.0293,0.0066</t>
-  </si>
-  <si>
-    <t>0.0062,0.9856,0.0216,0.0009</t>
-  </si>
-  <si>
-    <t>0.0061,0.9746,0.0670,0.0004</t>
-  </si>
-  <si>
-    <t>0.3387,0.0374,0.5795,0.0031</t>
-  </si>
-  <si>
-    <t>0.0296,0.8541,0.2542,0.0022</t>
-  </si>
-  <si>
-    <t>0.3576,0.0275,0.6096,0.0046</t>
-  </si>
-  <si>
-    <t>0.0303,0.6687,0.5274,0.0021</t>
-  </si>
-  <si>
-    <t>0.0006,0.9981,0.0061,0.0000</t>
-  </si>
-  <si>
-    <t>0.0509,0.1732,0.8065,0.0032</t>
-  </si>
-  <si>
-    <t>0.3709,0.5198,0.0967,0.0221</t>
-  </si>
-  <si>
-    <t>0.0100,0.9787,0.0254,0.0010</t>
-  </si>
-  <si>
-    <t>0.0118,0.9709,0.0421,0.0008</t>
-  </si>
-  <si>
-    <t>0.0034,0.9919,0.0117,0.0003</t>
-  </si>
-  <si>
-    <t>0.0005,0.4296,0.9845,0.0001</t>
-  </si>
-  <si>
-    <t>0.0098,0.1464,0.9374,0.0006</t>
-  </si>
-  <si>
-    <t>0.1417,0.0799,0.7330,0.0056</t>
-  </si>
-  <si>
-    <t>0.3991,0.0156,0.6110,0.0036</t>
-  </si>
-  <si>
-    <t>0.0143,0.4915,0.8140,0.0015</t>
-  </si>
-  <si>
-    <t>0.0959,0.1860,0.6494,0.0022</t>
-  </si>
-  <si>
-    <t>0.1358,0.8419,0.0400,0.0124</t>
-  </si>
-  <si>
-    <t>0.2739,0.6577,0.0416,0.0367</t>
-  </si>
-  <si>
-    <t>0.3458,0.5781,0.0395,0.0351</t>
-  </si>
-  <si>
-    <t>0.0013,0.1060,0.9913,0.0004</t>
-  </si>
-  <si>
-    <t>0.2717,0.6825,0.0400,0.0250</t>
-  </si>
-  <si>
-    <t>0.2119,0.7375,0.0330,0.0289</t>
-  </si>
-  <si>
-    <t>0.1863,0.7919,0.0393,0.0163</t>
-  </si>
-  <si>
-    <t>0.0007,0.9830,0.2693,0.0001</t>
-  </si>
-  <si>
-    <t>0.0002,0.0565,0.9980,0.0000</t>
-  </si>
-  <si>
-    <t>0.0141,0.5437,0.7116,0.0009</t>
-  </si>
-  <si>
-    <t>0.0111,0.6350,0.7016,0.0009</t>
-  </si>
-  <si>
-    <t>0.0025,0.0333,0.9903,0.0002</t>
-  </si>
-  <si>
-    <t>0.0084,0.9800,0.0294,0.0010</t>
-  </si>
-  <si>
-    <t>0.0001,0.9997,0.0007,0.0000</t>
-  </si>
-  <si>
-    <t>0.2503,0.0655,0.6314,0.0037</t>
-  </si>
-  <si>
-    <t>0.1596,0.6434,0.2050,0.0061</t>
-  </si>
-  <si>
-    <t>0.0013,0.4871,0.9737,0.0003</t>
-  </si>
-  <si>
-    <t>0.0016,0.9446,0.5330,0.0002</t>
-  </si>
-  <si>
-    <t>0.0346,0.7181,0.3647,0.0016</t>
-  </si>
-  <si>
-    <t>0.0007,0.9968,0.0162,0.0000</t>
-  </si>
-  <si>
-    <t>0.0006,0.9862,0.2745,0.0001</t>
-  </si>
-  <si>
-    <t>0.3551,0.5169,0.0911,0.0382</t>
-  </si>
-  <si>
-    <t>0.1462,0.5071,0.0130,0.4024</t>
-  </si>
-  <si>
-    <t>0.1578,0.3477,0.0157,0.5825</t>
-  </si>
-  <si>
-    <t>0.2958,0.5416,0.0431,0.0934</t>
-  </si>
-  <si>
-    <t>0.2951,0.5393,0.0474,0.0857</t>
-  </si>
-  <si>
-    <t>0.2334,0.5739,0.0465,0.1657</t>
-  </si>
-  <si>
-    <t>0.0079,0.9572,0.1388,0.0007</t>
-  </si>
-  <si>
-    <t>0.0019,0.9677,0.3217,0.0003</t>
-  </si>
-  <si>
-    <t>0.0088,0.8408,0.5233,0.0010</t>
-  </si>
-  <si>
-    <t>0.0070,0.8629,0.4770,0.0009</t>
-  </si>
-  <si>
-    <t>0.0016,0.9794,0.2056,0.0001</t>
-  </si>
-  <si>
-    <t>0.0031,0.9665,0.2010,0.0004</t>
-  </si>
-  <si>
-    <t>0.4100,0.5460,0.0504,0.0180</t>
-  </si>
-  <si>
-    <t>0.2258,0.7323,0.0359,0.0230</t>
-  </si>
-  <si>
-    <t>0.2576,0.6856,0.0369,0.0305</t>
-  </si>
-  <si>
-    <t>0.2287,0.7214,0.0406,0.0299</t>
-  </si>
-  <si>
-    <t>0.2674,0.6945,0.0429,0.0225</t>
-  </si>
-  <si>
-    <t>0.2419,0.6907,0.0403,0.0364</t>
-  </si>
-  <si>
-    <t>0.2380,0.6859,0.0344,0.0378</t>
-  </si>
-  <si>
-    <t>0.1341,0.8406,0.0343,0.0173</t>
-  </si>
-  <si>
-    <t>0.2964,0.5227,0.0210,0.0804</t>
-  </si>
-  <si>
-    <t>0.3402,0.5921,0.0379,0.0300</t>
-  </si>
-  <si>
-    <t>0.3484,0.4898,0.0293,0.0814</t>
-  </si>
-  <si>
-    <t>0.3953,0.4718,0.0260,0.0483</t>
-  </si>
-  <si>
-    <t>0.3526,0.4942,0.0266,0.0694</t>
-  </si>
-  <si>
-    <t>0.2180,0.7202,0.0352,0.0361</t>
-  </si>
-  <si>
-    <t>0.2792,0.6440,0.0297,0.0370</t>
-  </si>
-  <si>
-    <t>0.4546,0.3021,0.0225,0.0961</t>
-  </si>
-  <si>
-    <t>0.0001,0.0374,0.9991,0.0000</t>
-  </si>
-  <si>
-    <t>0.4688,0.0296,0.5014,0.0025</t>
-  </si>
-  <si>
-    <t>0.1622,0.7551,0.0965,0.0062</t>
-  </si>
-  <si>
-    <t>0.3160,0.0712,0.5238,0.0031</t>
-  </si>
-  <si>
-    <t>0.0099,0.9818,0.0150,0.0016</t>
-  </si>
-  <si>
-    <t>0.0077,0.9852,0.0134,0.0016</t>
-  </si>
-  <si>
-    <t>0.0134,0.9772,0.0154,0.0022</t>
-  </si>
-  <si>
-    <t>0.0285,0.9549,0.0263,0.0044</t>
-  </si>
-  <si>
-    <t>0.0234,0.9614,0.0250,0.0039</t>
-  </si>
-  <si>
-    <t>0.0047,0.9911,0.0074,0.0010</t>
-  </si>
-  <si>
-    <t>0.0408,0.9423,0.0254,0.0054</t>
-  </si>
-  <si>
-    <t>0.2551,0.5416,0.1641,0.0075</t>
-  </si>
-  <si>
-    <t>0.3293,0.3020,0.2881,0.0049</t>
-  </si>
-  <si>
-    <t>0.1115,0.8116,0.0777,0.0041</t>
-  </si>
-  <si>
-    <t>0.1825,0.7250,0.0920,0.0082</t>
-  </si>
-  <si>
-    <t>0.2597,0.5894,0.1358,0.0126</t>
-  </si>
-  <si>
-    <t>0.0020,0.9948,0.0099,0.0002</t>
-  </si>
-  <si>
-    <t>0.0042,0.9907,0.0123,0.0004</t>
-  </si>
-  <si>
-    <t>0.0206,0.9680,0.0185,0.0020</t>
-  </si>
-  <si>
-    <t>0.0006,0.9930,0.1240,0.0001</t>
-  </si>
-  <si>
-    <t>0.0067,0.9837,0.0233,0.0006</t>
-  </si>
-  <si>
-    <t>0.1335,0.8391,0.0464,0.0077</t>
-  </si>
-  <si>
-    <t>0.0704,0.9006,0.0444,0.0060</t>
-  </si>
-  <si>
-    <t>0.1066,0.8650,0.0462,0.0117</t>
-  </si>
-  <si>
-    <t>0.3022,0.5979,0.0352,0.0493</t>
-  </si>
-  <si>
-    <t>0.2581,0.6997,0.0376,0.0230</t>
-  </si>
-  <si>
-    <t>0.1496,0.8335,0.0344,0.0113</t>
-  </si>
-  <si>
-    <t>0.3494,0.5697,0.0358,0.0346</t>
-  </si>
-  <si>
-    <t>0.1375,0.8329,0.0469,0.0148</t>
-  </si>
-  <si>
-    <t>0.2322,0.7352,0.0452,0.0184</t>
-  </si>
-  <si>
-    <t>0.2900,0.6480,0.0347,0.0298</t>
-  </si>
-  <si>
-    <t>0.0140,0.8837,0.2326,0.0009</t>
-  </si>
-  <si>
-    <t>0.0393,0.3658,0.6529,0.0011</t>
-  </si>
-  <si>
-    <t>0.0266,0.6960,0.5443,0.0025</t>
-  </si>
-  <si>
-    <t>0.0481,0.5971,0.4853,0.0025</t>
-  </si>
-  <si>
-    <t>0.3311,0.4510,0.1354,0.0052</t>
-  </si>
-  <si>
-    <t>0.2457,0.6323,0.0983,0.0066</t>
-  </si>
-  <si>
-    <t>0.2540,0.3490,0.3391,0.0053</t>
-  </si>
-  <si>
-    <t>0.3394,0.3690,0.1922,0.0044</t>
-  </si>
-  <si>
-    <t>0.2837,0.6229,0.0530,0.0549</t>
-  </si>
-  <si>
-    <t>0.0689,0.1123,0.0054,0.9094</t>
-  </si>
-  <si>
-    <t>0.1433,0.3732,0.0163,0.6189</t>
-  </si>
-  <si>
-    <t>0.3790,0.3750,0.0562,0.1201</t>
-  </si>
-  <si>
-    <t>0.0002,0.9710,0.7482,0.0000</t>
-  </si>
-  <si>
-    <t>0.1751,0.7665,0.0271,0.0345</t>
-  </si>
-  <si>
-    <t>0.0387,0.9427,0.0291,0.0063</t>
-  </si>
-  <si>
-    <t>0.3339,0.6094,0.0463,0.0244</t>
-  </si>
-  <si>
-    <t>0.1552,0.8154,0.0504,0.0139</t>
-  </si>
-  <si>
-    <t>0.3127,0.6444,0.0613,0.0135</t>
-  </si>
-  <si>
-    <t>0.6650,0.1050,0.0867,0.0392</t>
-  </si>
-  <si>
-    <t>0.4200,0.5056,0.0587,0.0276</t>
-  </si>
-  <si>
-    <t>0.0055,0.3003,0.9606,0.0026</t>
-  </si>
-  <si>
-    <t>0.7744,0.0773,0.0804,0.0139</t>
-  </si>
-  <si>
-    <t>0.6533,0.1748,0.0662,0.0289</t>
-  </si>
-  <si>
-    <t>0.0251,0.9576,0.0311,0.0028</t>
-  </si>
-  <si>
-    <t>0.1985,0.7644,0.0636,0.0154</t>
-  </si>
-  <si>
-    <t>0.2054,0.7194,0.0981,0.0107</t>
-  </si>
-  <si>
-    <t>0.0368,0.9452,0.0307,0.0035</t>
-  </si>
-  <si>
-    <t>0.1798,0.7772,0.0698,0.0093</t>
-  </si>
-  <si>
-    <t>0.1237,0.8423,0.0577,0.0094</t>
-  </si>
-  <si>
-    <t>0.2214,0.7335,0.0341,0.0246</t>
-  </si>
-  <si>
-    <t>0.2732,0.6848,0.0485,0.0216</t>
-  </si>
-  <si>
-    <t>0.3429,0.6114,0.0385,0.0210</t>
-  </si>
-  <si>
-    <t>0.3250,0.6096,0.0500,0.0295</t>
-  </si>
-  <si>
-    <t>0.3454,0.5936,0.0474,0.0274</t>
-  </si>
-  <si>
-    <t>0.1463,0.8137,0.0326,0.0292</t>
-  </si>
-  <si>
-    <t>0.3481,0.5486,0.0352,0.0462</t>
-  </si>
-  <si>
-    <t>0.3184,0.6476,0.0356,0.0194</t>
-  </si>
-  <si>
-    <t>0.0332,0.9520,0.0226,0.0031</t>
-  </si>
-  <si>
-    <t>0.0773,0.8972,0.0314,0.0166</t>
-  </si>
-  <si>
-    <t>0.1439,0.8277,0.0502,0.0091</t>
-  </si>
-  <si>
-    <t>0.1606,0.5344,0.3474,0.0094</t>
-  </si>
-  <si>
-    <t>0.1669,0.8145,0.0374,0.0122</t>
-  </si>
-  <si>
-    <t>0.1885,0.7959,0.0378,0.0112</t>
-  </si>
-  <si>
-    <t>0.2262,0.7485,0.0365,0.0160</t>
-  </si>
-  <si>
-    <t>0.0679,0.9139,0.0240,0.0109</t>
-  </si>
-  <si>
-    <t>0.0000,0.5577,0.9974,0.0000</t>
-  </si>
-  <si>
-    <t>0.2211,0.7428,0.0548,0.0182</t>
-  </si>
-  <si>
-    <t>0.0285,0.0537,0.9130,0.0006</t>
-  </si>
-  <si>
-    <t>0.0154,0.4434,0.8191,0.0017</t>
-  </si>
-  <si>
-    <t>0.1880,0.3591,0.4572,0.0071</t>
-  </si>
-  <si>
-    <t>0.0002,0.1740,0.9962,0.0000</t>
-  </si>
-  <si>
-    <t>0.0180,0.0970,0.9343,0.0010</t>
-  </si>
-  <si>
-    <t>0.0138,0.0108,0.9750,0.0005</t>
-  </si>
-  <si>
-    <t>0.1363,0.0853,0.7325,0.0046</t>
-  </si>
-  <si>
-    <t>0.3325,0.3845,0.2141,0.0075</t>
-  </si>
-  <si>
-    <t>0.1614,0.0816,0.7191,0.0053</t>
-  </si>
-  <si>
-    <t>0.3003,0.3434,0.2731,0.0046</t>
-  </si>
-  <si>
-    <t>0.1692,0.6419,0.1248,0.0029</t>
-  </si>
-  <si>
-    <t>0.1206,0.7781,0.1060,0.0050</t>
-  </si>
-  <si>
-    <t>0.1522,0.7559,0.1038,0.0073</t>
-  </si>
-  <si>
-    <t>0.1797,0.7166,0.1150,0.0080</t>
-  </si>
-  <si>
-    <t>0.2905,0.4643,0.1909,0.0058</t>
-  </si>
-  <si>
-    <t>0.0401,0.9457,0.0195,0.0055</t>
-  </si>
-  <si>
-    <t>0.0573,0.9262,0.0246,0.0054</t>
-  </si>
-  <si>
-    <t>0.0288,0.9577,0.0198,0.0037</t>
-  </si>
-  <si>
-    <t>0.1083,0.8608,0.0284,0.0240</t>
-  </si>
-  <si>
-    <t>0.1098,0.8700,0.0270,0.0144</t>
-  </si>
-  <si>
-    <t>0.2470,0.5635,0.1280,0.0035</t>
-  </si>
-  <si>
-    <t>0.2666,0.6203,0.1025,0.0066</t>
-  </si>
-  <si>
-    <t>0.2237,0.6409,0.1181,0.0066</t>
-  </si>
-  <si>
-    <t>0.3894,0.1554,0.3621,0.0042</t>
-  </si>
-  <si>
-    <t>0.2069,0.5646,0.1591,0.0034</t>
-  </si>
-  <si>
-    <t>0.0419,0.5571,0.5998,0.0038</t>
-  </si>
-  <si>
-    <t>0.0715,0.2621,0.6851,0.0031</t>
-  </si>
-  <si>
-    <t>0.0878,0.6112,0.2770,0.0022</t>
-  </si>
-  <si>
-    <t>0.0691,0.6407,0.2917,0.0023</t>
-  </si>
-  <si>
-    <t>0.0718,0.4684,0.4132,0.0018</t>
-  </si>
-  <si>
-    <t>0.2616,0.6399,0.0236,0.0488</t>
-  </si>
-  <si>
-    <t>0.1871,0.7733,0.0309,0.0268</t>
-  </si>
-  <si>
-    <t>0.1082,0.8560,0.0254,0.0276</t>
-  </si>
-  <si>
-    <t>0.1876,0.7730,0.0350,0.0259</t>
-  </si>
-  <si>
-    <t>0.1837,0.7561,0.0258,0.0400</t>
-  </si>
-  <si>
-    <t>0.1839,0.7493,0.0243,0.0382</t>
-  </si>
-  <si>
-    <t>0.2272,0.7130,0.0320,0.0338</t>
-  </si>
-  <si>
-    <t>0.2383,0.7066,0.0320,0.0284</t>
-  </si>
-  <si>
-    <t>0.0772,0.2777,0.7425,0.0079</t>
-  </si>
-  <si>
-    <t>0.1392,0.8028,0.0711,0.0064</t>
-  </si>
-  <si>
-    <t>0.1104,0.8524,0.0578,0.0086</t>
-  </si>
-  <si>
-    <t>0.1023,0.1447,0.6979,0.0024</t>
-  </si>
-  <si>
-    <t>0.0013,0.3865,0.9697,0.0002</t>
-  </si>
-  <si>
-    <t>0.1240,0.2415,0.5908,0.0049</t>
-  </si>
-  <si>
-    <t>0.0022,0.0323,0.9912,0.0001</t>
-  </si>
-  <si>
-    <t>0.1249,0.2488,0.6049,0.0046</t>
-  </si>
-  <si>
-    <t>0.0000,0.0221,0.9997,0.0000</t>
-  </si>
-  <si>
-    <t>0.1988,0.0497,0.7000,0.0040</t>
-  </si>
-  <si>
-    <t>0.0258,0.5129,0.7043,0.0023</t>
-  </si>
-  <si>
-    <t>0.4811,0.1574,0.2506,0.0040</t>
-  </si>
-  <si>
-    <t>0.2925,0.1538,0.4406,0.0042</t>
-  </si>
-  <si>
-    <t>0.2651,0.6102,0.1096,0.0089</t>
-  </si>
-  <si>
-    <t>0.2030,0.7510,0.0289,0.0284</t>
-  </si>
-  <si>
-    <t>0.2597,0.6964,0.0410,0.0234</t>
-  </si>
-  <si>
-    <t>0.3427,0.5829,0.0291,0.0290</t>
-  </si>
-  <si>
-    <t>0.2516,0.7159,0.0419,0.0182</t>
-  </si>
-  <si>
-    <t>0.1822,0.7244,0.0228,0.0667</t>
-  </si>
-  <si>
-    <t>0.3558,0.5714,0.0403,0.0334</t>
-  </si>
-  <si>
-    <t>0.2017,0.7412,0.0272,0.0321</t>
-  </si>
-  <si>
-    <t>0.2550,0.6509,0.0304,0.0466</t>
-  </si>
-  <si>
-    <t>0.1255,0.5875,0.2387,0.0038</t>
-  </si>
-  <si>
-    <t>0.0025,0.2068,0.9724,0.0002</t>
-  </si>
-  <si>
-    <t>0.0070,0.5481,0.8498,0.0009</t>
-  </si>
-  <si>
-    <t>0.3845,0.2448,0.2508,0.0038</t>
-  </si>
-  <si>
-    <t>0.0069,0.1526,0.9534,0.0005</t>
-  </si>
-  <si>
-    <t>0.5463,0.0633,0.3806,0.0057</t>
-  </si>
-  <si>
-    <t>0.1039,0.5193,0.3421,0.0020</t>
-  </si>
-  <si>
-    <t>0.1518,0.0176,0.8122,0.0024</t>
-  </si>
-  <si>
-    <t>0.5999,0.2407,0.0498,0.0293</t>
-  </si>
-  <si>
-    <t>0.0977,0.7592,0.0198,0.2407</t>
-  </si>
-  <si>
-    <t>0.2107,0.6520,0.0266,0.0901</t>
-  </si>
-  <si>
-    <t>0.3163,0.1781,0.0221,0.3381</t>
-  </si>
-  <si>
-    <t>0.0675,0.3140,0.0052,0.8372</t>
-  </si>
-  <si>
-    <t>0.5916,0.1862,0.1713,0.0153</t>
+    <t>0.0929,0.8708,0.0568,0.0068</t>
+  </si>
+  <si>
+    <t>0.2938,0.2749,0.0196,0.2861</t>
+  </si>
+  <si>
+    <t>0.2424,0.7245,0.0540,0.0156</t>
+  </si>
+  <si>
+    <t>0.6532,0.0931,0.2109,0.0110</t>
+  </si>
+  <si>
+    <t>0.3321,0.5153,0.0199,0.0618</t>
+  </si>
+  <si>
+    <t>0.3295,0.5168,0.0199,0.0552</t>
+  </si>
+  <si>
+    <t>0.2340,0.7458,0.0376,0.0140</t>
+  </si>
+  <si>
+    <t>0.4708,0.3950,0.0338,0.0440</t>
+  </si>
+  <si>
+    <t>0.2414,0.6697,0.0280,0.0438</t>
+  </si>
+  <si>
+    <t>0.2439,0.7055,0.0361,0.0281</t>
+  </si>
+  <si>
+    <t>0.3289,0.5865,0.0340,0.0371</t>
+  </si>
+  <si>
+    <t>0.3266,0.5650,0.0261,0.0450</t>
+  </si>
+  <si>
+    <t>0.1873,0.7083,0.0995,0.0048</t>
+  </si>
+  <si>
+    <t>0.1278,0.5002,0.3663,0.0043</t>
+  </si>
+  <si>
+    <t>0.0834,0.7790,0.1754,0.0052</t>
+  </si>
+  <si>
+    <t>0.2992,0.3205,0.2644,0.0041</t>
+  </si>
+  <si>
+    <t>0.1841,0.7332,0.0855,0.0064</t>
+  </si>
+  <si>
+    <t>0.0194,0.9649,0.0280,0.0015</t>
+  </si>
+  <si>
+    <t>0.0100,0.9795,0.0210,0.0013</t>
+  </si>
+  <si>
+    <t>0.0156,0.9736,0.0187,0.0021</t>
+  </si>
+  <si>
+    <t>0.0184,0.9661,0.0280,0.0025</t>
+  </si>
+  <si>
+    <t>0.0042,0.9898,0.0153,0.0006</t>
+  </si>
+  <si>
+    <t>0.1729,0.7035,0.1202,0.0072</t>
+  </si>
+  <si>
+    <t>0.1589,0.5955,0.1982,0.0031</t>
+  </si>
+  <si>
+    <t>0.1527,0.0433,0.7570,0.0024</t>
+  </si>
+  <si>
+    <t>0.3389,0.3087,0.2241,0.0036</t>
+  </si>
+  <si>
+    <t>0.3446,0.0250,0.6269,0.0039</t>
+  </si>
+  <si>
+    <t>0.3988,0.0249,0.5838,0.0040</t>
+  </si>
+  <si>
+    <t>0.0482,0.1057,0.8260,0.0012</t>
+  </si>
+  <si>
+    <t>0.0232,0.9569,0.0382,0.0031</t>
+  </si>
+  <si>
+    <t>0.2667,0.5859,0.1347,0.0066</t>
+  </si>
+  <si>
+    <t>0.0000,0.4486,0.9984,0.0000</t>
+  </si>
+  <si>
+    <t>0.0251,0.9472,0.0489,0.0009</t>
+  </si>
+  <si>
+    <t>0.2149,0.7311,0.0774,0.0272</t>
+  </si>
+  <si>
+    <t>0.1351,0.7993,0.0946,0.0103</t>
+  </si>
+  <si>
+    <t>0.0689,0.9106,0.0317,0.0063</t>
+  </si>
+  <si>
+    <t>0.0112,0.9740,0.0359,0.0011</t>
+  </si>
+  <si>
+    <t>0.0031,0.9647,0.2303,0.0004</t>
+  </si>
+  <si>
+    <t>0.2197,0.1116,0.5398,0.0038</t>
+  </si>
+  <si>
+    <t>0.0987,0.4914,0.4225,0.0043</t>
+  </si>
+  <si>
+    <t>0.5190,0.0267,0.4781,0.0035</t>
+  </si>
+  <si>
+    <t>0.0501,0.7714,0.2490,0.0016</t>
+  </si>
+  <si>
+    <t>0.0025,0.9936,0.0107,0.0001</t>
+  </si>
+  <si>
+    <t>0.0225,0.1258,0.9109,0.0017</t>
+  </si>
+  <si>
+    <t>0.3184,0.6016,0.0633,0.0270</t>
+  </si>
+  <si>
+    <t>0.0106,0.9800,0.0186,0.0011</t>
+  </si>
+  <si>
+    <t>0.0036,0.9916,0.0117,0.0003</t>
+  </si>
+  <si>
+    <t>0.0075,0.9856,0.0133,0.0005</t>
+  </si>
+  <si>
+    <t>0.0032,0.0278,0.9883,0.0004</t>
+  </si>
+  <si>
+    <t>0.0304,0.0688,0.9083,0.0016</t>
+  </si>
+  <si>
+    <t>0.3263,0.1524,0.4189,0.0061</t>
+  </si>
+  <si>
+    <t>0.3629,0.0136,0.6467,0.0035</t>
+  </si>
+  <si>
+    <t>0.0049,0.5960,0.8865,0.0007</t>
+  </si>
+  <si>
+    <t>0.0202,0.1601,0.8862,0.0009</t>
+  </si>
+  <si>
+    <t>0.1753,0.8028,0.0415,0.0142</t>
+  </si>
+  <si>
+    <t>0.3076,0.6304,0.0487,0.0314</t>
+  </si>
+  <si>
+    <t>0.2728,0.6537,0.0285,0.0376</t>
+  </si>
+  <si>
+    <t>0.0026,0.2554,0.9786,0.0009</t>
+  </si>
+  <si>
+    <t>0.2786,0.6719,0.0400,0.0255</t>
+  </si>
+  <si>
+    <t>0.2052,0.6905,0.0220,0.0615</t>
+  </si>
+  <si>
+    <t>0.2426,0.7094,0.0394,0.0299</t>
+  </si>
+  <si>
+    <t>0.0025,0.9095,0.5629,0.0004</t>
+  </si>
+  <si>
+    <t>0.0003,0.0475,0.9976,0.0001</t>
+  </si>
+  <si>
+    <t>0.0137,0.1597,0.9153,0.0008</t>
+  </si>
+  <si>
+    <t>0.0025,0.9598,0.2972,0.0003</t>
+  </si>
+  <si>
+    <t>0.0034,0.0269,0.9886,0.0002</t>
+  </si>
+  <si>
+    <t>0.0077,0.9807,0.0300,0.0008</t>
+  </si>
+  <si>
+    <t>0.0001,0.9998,0.0004,0.0000</t>
+  </si>
+  <si>
+    <t>0.2659,0.1159,0.5608,0.0062</t>
+  </si>
+  <si>
+    <t>0.1807,0.6871,0.1249,0.0049</t>
+  </si>
+  <si>
+    <t>0.0020,0.8034,0.8905,0.0005</t>
+  </si>
+  <si>
+    <t>0.0007,0.9796,0.3614,0.0001</t>
+  </si>
+  <si>
+    <t>0.0137,0.8171,0.4300,0.0011</t>
+  </si>
+  <si>
+    <t>0.0007,0.9976,0.0078,0.0000</t>
+  </si>
+  <si>
+    <t>0.0004,0.9910,0.2217,0.0000</t>
+  </si>
+  <si>
+    <t>0.6663,0.1046,0.1826,0.0136</t>
+  </si>
+  <si>
+    <t>0.2269,0.2331,0.0156,0.4672</t>
+  </si>
+  <si>
+    <t>0.2800,0.0859,0.0133,0.5260</t>
+  </si>
+  <si>
+    <t>0.3003,0.5212,0.0412,0.1001</t>
+  </si>
+  <si>
+    <t>0.1506,0.7760,0.0506,0.0517</t>
+  </si>
+  <si>
+    <t>0.3533,0.3664,0.0402,0.1608</t>
+  </si>
+  <si>
+    <t>0.0025,0.9645,0.2926,0.0003</t>
+  </si>
+  <si>
+    <t>0.0015,0.9597,0.4711,0.0002</t>
+  </si>
+  <si>
+    <t>0.0079,0.8383,0.5040,0.0008</t>
+  </si>
+  <si>
+    <t>0.0453,0.5997,0.4457,0.0024</t>
+  </si>
+  <si>
+    <t>0.0014,0.9799,0.2101,0.0001</t>
+  </si>
+  <si>
+    <t>0.0075,0.9005,0.3783,0.0008</t>
+  </si>
+  <si>
+    <t>0.2911,0.6472,0.0369,0.0285</t>
+  </si>
+  <si>
+    <t>0.2395,0.7250,0.0328,0.0197</t>
+  </si>
+  <si>
+    <t>0.2471,0.7182,0.0336,0.0210</t>
+  </si>
+  <si>
+    <t>0.2764,0.6339,0.0358,0.0436</t>
+  </si>
+  <si>
+    <t>0.2417,0.7148,0.0435,0.0242</t>
+  </si>
+  <si>
+    <t>0.3405,0.5101,0.0260,0.0644</t>
+  </si>
+  <si>
+    <t>0.3070,0.6175,0.0421,0.0328</t>
+  </si>
+  <si>
+    <t>0.1943,0.7659,0.0307,0.0247</t>
+  </si>
+  <si>
+    <t>0.2522,0.5496,0.0241,0.1227</t>
+  </si>
+  <si>
+    <t>0.3880,0.5433,0.0340,0.0264</t>
+  </si>
+  <si>
+    <t>0.3798,0.5008,0.0280,0.0487</t>
+  </si>
+  <si>
+    <t>0.4031,0.4734,0.0297,0.0458</t>
+  </si>
+  <si>
+    <t>0.3764,0.4983,0.0270,0.0518</t>
+  </si>
+  <si>
+    <t>0.3114,0.6112,0.0324,0.0374</t>
+  </si>
+  <si>
+    <t>0.1896,0.7461,0.0230,0.0357</t>
+  </si>
+  <si>
+    <t>0.4426,0.3396,0.0295,0.0935</t>
+  </si>
+  <si>
+    <t>0.0002,0.0499,0.9979,0.0001</t>
+  </si>
+  <si>
+    <t>0.2589,0.0392,0.6452,0.0023</t>
+  </si>
+  <si>
+    <t>0.3654,0.3687,0.2013,0.0055</t>
+  </si>
+  <si>
+    <t>0.3056,0.0829,0.5312,0.0032</t>
+  </si>
+  <si>
+    <t>0.0078,0.9852,0.0129,0.0019</t>
+  </si>
+  <si>
+    <t>0.0070,0.9863,0.0128,0.0019</t>
+  </si>
+  <si>
+    <t>0.0240,0.9649,0.0151,0.0034</t>
+  </si>
+  <si>
+    <t>0.0336,0.9481,0.0285,0.0046</t>
+  </si>
+  <si>
+    <t>0.0089,0.9832,0.0144,0.0020</t>
+  </si>
+  <si>
+    <t>0.0027,0.9938,0.0081,0.0007</t>
+  </si>
+  <si>
+    <t>0.0308,0.9507,0.0290,0.0040</t>
+  </si>
+  <si>
+    <t>0.1982,0.6544,0.1118,0.0047</t>
+  </si>
+  <si>
+    <t>0.2337,0.1226,0.5613,0.0039</t>
+  </si>
+  <si>
+    <t>0.2732,0.5238,0.1439,0.0057</t>
+  </si>
+  <si>
+    <t>0.0779,0.8714,0.0783,0.0052</t>
+  </si>
+  <si>
+    <t>0.1032,0.8472,0.0773,0.0086</t>
+  </si>
+  <si>
+    <t>0.0060,0.9872,0.0154,0.0004</t>
+  </si>
+  <si>
+    <t>0.0017,0.9964,0.0046,0.0002</t>
+  </si>
+  <si>
+    <t>0.0570,0.9220,0.0342,0.0048</t>
+  </si>
+  <si>
+    <t>0.0009,0.9930,0.0738,0.0001</t>
+  </si>
+  <si>
+    <t>0.0029,0.9916,0.0182,0.0004</t>
+  </si>
+  <si>
+    <t>0.0920,0.8778,0.0468,0.0061</t>
+  </si>
+  <si>
+    <t>0.0730,0.8983,0.0444,0.0075</t>
+  </si>
+  <si>
+    <t>0.1147,0.8458,0.0644,0.0113</t>
+  </si>
+  <si>
+    <t>0.2544,0.6671,0.0352,0.0403</t>
+  </si>
+  <si>
+    <t>0.2689,0.6657,0.0303,0.0314</t>
+  </si>
+  <si>
+    <t>0.1012,0.8799,0.0232,0.0136</t>
+  </si>
+  <si>
+    <t>0.2498,0.6704,0.0269,0.0418</t>
+  </si>
+  <si>
+    <t>0.1838,0.7794,0.0605,0.0140</t>
+  </si>
+  <si>
+    <t>0.2999,0.6578,0.0404,0.0224</t>
+  </si>
+  <si>
+    <t>0.3332,0.6258,0.0502,0.0201</t>
+  </si>
+  <si>
+    <t>0.0126,0.7538,0.5361,0.0011</t>
+  </si>
+  <si>
+    <t>0.0155,0.6075,0.6445,0.0010</t>
+  </si>
+  <si>
+    <t>0.0165,0.6680,0.6745,0.0021</t>
+  </si>
+  <si>
+    <t>0.0401,0.3813,0.6938,0.0021</t>
+  </si>
+  <si>
+    <t>0.2406,0.6269,0.1006,0.0057</t>
+  </si>
+  <si>
+    <t>0.1207,0.7503,0.1385,0.0051</t>
+  </si>
+  <si>
+    <t>0.1986,0.2477,0.4818,0.0048</t>
+  </si>
+  <si>
+    <t>0.1641,0.7370,0.0967,0.0050</t>
+  </si>
+  <si>
+    <t>0.3864,0.4716,0.0587,0.0707</t>
+  </si>
+  <si>
+    <t>0.0489,0.2968,0.0052,0.9022</t>
+  </si>
+  <si>
+    <t>0.1278,0.1908,0.0139,0.7725</t>
+  </si>
+  <si>
+    <t>0.3255,0.4547,0.0397,0.1210</t>
+  </si>
+  <si>
+    <t>0.0005,0.9615,0.6697,0.0001</t>
+  </si>
+  <si>
+    <t>0.1674,0.8005,0.0317,0.0207</t>
+  </si>
+  <si>
+    <t>0.0278,0.9567,0.0234,0.0055</t>
+  </si>
+  <si>
+    <t>0.2479,0.7155,0.0439,0.0209</t>
+  </si>
+  <si>
+    <t>0.1853,0.7815,0.0611,0.0137</t>
+  </si>
+  <si>
+    <t>0.2029,0.7493,0.0718,0.0115</t>
+  </si>
+  <si>
+    <t>0.6718,0.1374,0.1204,0.0176</t>
+  </si>
+  <si>
+    <t>0.3426,0.5921,0.0681,0.0290</t>
+  </si>
+  <si>
+    <t>0.0053,0.4215,0.9509,0.0034</t>
+  </si>
+  <si>
+    <t>0.7520,0.0875,0.1091,0.0127</t>
+  </si>
+  <si>
+    <t>0.7270,0.1394,0.0879,0.0117</t>
+  </si>
+  <si>
+    <t>0.0389,0.9340,0.0501,0.0040</t>
+  </si>
+  <si>
+    <t>0.2171,0.7384,0.0776,0.0121</t>
+  </si>
+  <si>
+    <t>0.1842,0.7666,0.0801,0.0106</t>
+  </si>
+  <si>
+    <t>0.0468,0.9320,0.0361,0.0036</t>
+  </si>
+  <si>
+    <t>0.3816,0.4633,0.1132,0.0058</t>
+  </si>
+  <si>
+    <t>0.1105,0.8611,0.0466,0.0089</t>
+  </si>
+  <si>
+    <t>0.3939,0.5129,0.0363,0.0333</t>
+  </si>
+  <si>
+    <t>0.2729,0.6381,0.0308,0.0414</t>
+  </si>
+  <si>
+    <t>0.2893,0.6710,0.0440,0.0210</t>
+  </si>
+  <si>
+    <t>0.3093,0.5901,0.0346,0.0475</t>
+  </si>
+  <si>
+    <t>0.3486,0.5989,0.0413,0.0237</t>
+  </si>
+  <si>
+    <t>0.1677,0.8044,0.0401,0.0187</t>
+  </si>
+  <si>
+    <t>0.4395,0.4843,0.0451,0.0291</t>
+  </si>
+  <si>
+    <t>0.3355,0.5717,0.0285,0.0388</t>
+  </si>
+  <si>
+    <t>0.0743,0.9022,0.0380,0.0056</t>
+  </si>
+  <si>
+    <t>0.0792,0.8967,0.0328,0.0146</t>
+  </si>
+  <si>
+    <t>0.0697,0.9025,0.0445,0.0075</t>
+  </si>
+  <si>
+    <t>0.2708,0.5815,0.1422,0.0091</t>
+  </si>
+  <si>
+    <t>0.1130,0.8741,0.0267,0.0072</t>
+  </si>
+  <si>
+    <t>0.2105,0.7681,0.0437,0.0128</t>
+  </si>
+  <si>
+    <t>0.1910,0.7719,0.0392,0.0215</t>
+  </si>
+  <si>
+    <t>0.1116,0.8611,0.0361,0.0166</t>
+  </si>
+  <si>
+    <t>0.0001,0.4901,0.9947,0.0000</t>
+  </si>
+  <si>
+    <t>0.2619,0.6992,0.0635,0.0140</t>
+  </si>
+  <si>
+    <t>0.0233,0.0694,0.9183,0.0005</t>
+  </si>
+  <si>
+    <t>0.0170,0.2404,0.8840,0.0012</t>
+  </si>
+  <si>
+    <t>0.1467,0.2022,0.6224,0.0050</t>
+  </si>
+  <si>
+    <t>0.0004,0.0995,0.9958,0.0001</t>
+  </si>
+  <si>
+    <t>0.0345,0.1438,0.8692,0.0019</t>
+  </si>
+  <si>
+    <t>0.0119,0.0331,0.9685,0.0006</t>
+  </si>
+  <si>
+    <t>0.0222,0.1118,0.9216,0.0019</t>
+  </si>
+  <si>
+    <t>0.1850,0.4191,0.3372,0.0053</t>
+  </si>
+  <si>
+    <t>0.4282,0.0598,0.4934,0.0077</t>
+  </si>
+  <si>
+    <t>0.2895,0.4772,0.1641,0.0049</t>
+  </si>
+  <si>
+    <t>0.1686,0.6516,0.1594,0.0048</t>
+  </si>
+  <si>
+    <t>0.0778,0.8102,0.1310,0.0038</t>
+  </si>
+  <si>
+    <t>0.2091,0.6626,0.1267,0.0093</t>
+  </si>
+  <si>
+    <t>0.2158,0.6906,0.1126,0.0127</t>
+  </si>
+  <si>
+    <t>0.1237,0.7611,0.1374,0.0065</t>
+  </si>
+  <si>
+    <t>0.0346,0.9521,0.0190,0.0046</t>
+  </si>
+  <si>
+    <t>0.0570,0.9218,0.0316,0.0055</t>
+  </si>
+  <si>
+    <t>0.0329,0.9523,0.0217,0.0041</t>
+  </si>
+  <si>
+    <t>0.1077,0.8562,0.0272,0.0296</t>
+  </si>
+  <si>
+    <t>0.1008,0.8765,0.0242,0.0170</t>
+  </si>
+  <si>
+    <t>0.1540,0.7180,0.0957,0.0026</t>
+  </si>
+  <si>
+    <t>0.2261,0.5997,0.1542,0.0063</t>
+  </si>
+  <si>
+    <t>0.1409,0.7882,0.0843,0.0058</t>
+  </si>
+  <si>
+    <t>0.3394,0.3721,0.1932,0.0045</t>
+  </si>
+  <si>
+    <t>0.2758,0.4744,0.1728,0.0046</t>
+  </si>
+  <si>
+    <t>0.0311,0.4873,0.7230,0.0031</t>
+  </si>
+  <si>
+    <t>0.1244,0.3419,0.4792,0.0039</t>
+  </si>
+  <si>
+    <t>0.1282,0.3427,0.4516,0.0033</t>
+  </si>
+  <si>
+    <t>0.1902,0.2000,0.4787,0.0033</t>
+  </si>
+  <si>
+    <t>0.0407,0.6169,0.3993,0.0016</t>
+  </si>
+  <si>
+    <t>0.2773,0.6278,0.0273,0.0462</t>
+  </si>
+  <si>
+    <t>0.1327,0.8380,0.0253,0.0225</t>
+  </si>
+  <si>
+    <t>0.1524,0.8128,0.0326,0.0237</t>
+  </si>
+  <si>
+    <t>0.2299,0.7282,0.0357,0.0252</t>
+  </si>
+  <si>
+    <t>0.1988,0.7584,0.0344,0.0277</t>
+  </si>
+  <si>
+    <t>0.2120,0.7180,0.0267,0.0377</t>
+  </si>
+  <si>
+    <t>0.1756,0.7639,0.0314,0.0423</t>
+  </si>
+  <si>
+    <t>0.3281,0.6251,0.0405,0.0212</t>
+  </si>
+  <si>
+    <t>0.1910,0.0804,0.6986,0.0077</t>
+  </si>
+  <si>
+    <t>0.1208,0.8311,0.0712,0.0081</t>
+  </si>
+  <si>
+    <t>0.0799,0.8887,0.0507,0.0054</t>
+  </si>
+  <si>
+    <t>0.0030,0.2195,0.9659,0.0002</t>
+  </si>
+  <si>
+    <t>0.0009,0.2180,0.9861,0.0002</t>
+  </si>
+  <si>
+    <t>0.1341,0.1132,0.7042,0.0061</t>
+  </si>
+  <si>
+    <t>0.0003,0.0253,0.9982,0.0000</t>
+  </si>
+  <si>
+    <t>0.1399,0.5069,0.3475,0.0049</t>
+  </si>
+  <si>
+    <t>0.0000,0.0237,0.9995,0.0000</t>
+  </si>
+  <si>
+    <t>0.2241,0.1054,0.5887,0.0051</t>
+  </si>
+  <si>
+    <t>0.0863,0.7843,0.1747,0.0050</t>
+  </si>
+  <si>
+    <t>0.4125,0.3686,0.1455,0.0077</t>
+  </si>
+  <si>
+    <t>0.3656,0.3165,0.2196,0.0059</t>
+  </si>
+  <si>
+    <t>0.3759,0.3959,0.1698,0.0071</t>
+  </si>
+  <si>
+    <t>0.1786,0.7825,0.0284,0.0255</t>
+  </si>
+  <si>
+    <t>0.3107,0.6115,0.0364,0.0340</t>
+  </si>
+  <si>
+    <t>0.2930,0.6028,0.0250,0.0445</t>
+  </si>
+  <si>
+    <t>0.1448,0.8047,0.0254,0.0338</t>
+  </si>
+  <si>
+    <t>0.3943,0.4569,0.0273,0.0540</t>
+  </si>
+  <si>
+    <t>0.2862,0.6430,0.0354,0.0337</t>
+  </si>
+  <si>
+    <t>0.1559,0.7980,0.0230,0.0304</t>
+  </si>
+  <si>
+    <t>0.2225,0.6707,0.0216,0.0553</t>
+  </si>
+  <si>
+    <t>0.0512,0.8348,0.1868,0.0039</t>
+  </si>
+  <si>
+    <t>0.0057,0.4641,0.8951,0.0006</t>
+  </si>
+  <si>
+    <t>0.0141,0.5456,0.7496,0.0014</t>
+  </si>
+  <si>
+    <t>0.1212,0.7703,0.0799,0.0016</t>
+  </si>
+  <si>
+    <t>0.0386,0.1292,0.8398,0.0013</t>
+  </si>
+  <si>
+    <t>0.2258,0.1415,0.5709,0.0065</t>
+  </si>
+  <si>
+    <t>0.1749,0.2453,0.4807,0.0030</t>
+  </si>
+  <si>
+    <t>0.3977,0.0127,0.6257,0.0024</t>
+  </si>
+  <si>
+    <t>0.4606,0.3357,0.0381,0.0556</t>
+  </si>
+  <si>
+    <t>0.1622,0.6128,0.0229,0.2695</t>
+  </si>
+  <si>
+    <t>0.2903,0.5414,0.0264,0.0783</t>
+  </si>
+  <si>
+    <t>0.5082,0.2145,0.0563,0.0990</t>
+  </si>
+  <si>
+    <t>0.0648,0.2536,0.0044,0.8627</t>
+  </si>
+  <si>
+    <t>0.5965,0.2073,0.1526,0.0108</t>
   </si>
 </sst>
 </file>
@@ -2009,7 +2009,7 @@
         <v>259</v>
       </c>
       <c r="C6" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D6" t="s">
         <v>268</v>
@@ -2107,7 +2107,7 @@
         <v>259</v>
       </c>
       <c r="C13" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D13" t="s">
         <v>275</v>
@@ -2261,7 +2261,7 @@
         <v>259</v>
       </c>
       <c r="C24" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D24" t="s">
         <v>286</v>
@@ -2275,7 +2275,7 @@
         <v>259</v>
       </c>
       <c r="C25" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D25" t="s">
         <v>287</v>
@@ -2499,7 +2499,7 @@
         <v>261</v>
       </c>
       <c r="C41" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="D41" t="s">
         <v>303</v>
@@ -2513,7 +2513,7 @@
         <v>261</v>
       </c>
       <c r="C42" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="D42" t="s">
         <v>304</v>
@@ -2527,7 +2527,7 @@
         <v>263</v>
       </c>
       <c r="C43" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D43" t="s">
         <v>305</v>
@@ -2653,7 +2653,7 @@
         <v>261</v>
       </c>
       <c r="C52" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="D52" t="s">
         <v>314</v>
@@ -2681,7 +2681,7 @@
         <v>261</v>
       </c>
       <c r="C54" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="D54" t="s">
         <v>316</v>
@@ -2807,7 +2807,7 @@
         <v>262</v>
       </c>
       <c r="C63" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D63" t="s">
         <v>325</v>
@@ -2835,7 +2835,7 @@
         <v>261</v>
       </c>
       <c r="C65" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="D65" t="s">
         <v>327</v>
@@ -2849,7 +2849,7 @@
         <v>263</v>
       </c>
       <c r="C66" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D66" t="s">
         <v>328</v>
@@ -2933,7 +2933,7 @@
         <v>261</v>
       </c>
       <c r="C72" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="D72" t="s">
         <v>334</v>
@@ -2947,7 +2947,7 @@
         <v>263</v>
       </c>
       <c r="C73" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D73" t="s">
         <v>335</v>
@@ -3003,7 +3003,7 @@
         <v>260</v>
       </c>
       <c r="C77" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="D77" t="s">
         <v>339</v>
@@ -3017,7 +3017,7 @@
         <v>260</v>
       </c>
       <c r="C78" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="D78" t="s">
         <v>340</v>
@@ -3073,7 +3073,7 @@
         <v>260</v>
       </c>
       <c r="C82" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="D82" t="s">
         <v>344</v>
@@ -3311,7 +3311,7 @@
         <v>259</v>
       </c>
       <c r="C99" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D99" t="s">
         <v>361</v>
@@ -3423,7 +3423,7 @@
         <v>259</v>
       </c>
       <c r="C107" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="D107" t="s">
         <v>369</v>
@@ -3563,7 +3563,7 @@
         <v>261</v>
       </c>
       <c r="C117" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D117" t="s">
         <v>379</v>
@@ -3829,7 +3829,7 @@
         <v>263</v>
       </c>
       <c r="C136" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D136" t="s">
         <v>398</v>
@@ -3843,7 +3843,7 @@
         <v>261</v>
       </c>
       <c r="C137" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="D137" t="s">
         <v>399</v>
@@ -3871,7 +3871,7 @@
         <v>261</v>
       </c>
       <c r="C139" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="D139" t="s">
         <v>401</v>
@@ -3885,7 +3885,7 @@
         <v>259</v>
       </c>
       <c r="C140" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D140" t="s">
         <v>402</v>
@@ -3927,7 +3927,7 @@
         <v>259</v>
       </c>
       <c r="C143" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D143" t="s">
         <v>405</v>
@@ -3941,7 +3941,7 @@
         <v>260</v>
       </c>
       <c r="C144" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="D144" t="s">
         <v>406</v>
@@ -4207,7 +4207,7 @@
         <v>259</v>
       </c>
       <c r="C163" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="D163" t="s">
         <v>425</v>
@@ -4319,7 +4319,7 @@
         <v>259</v>
       </c>
       <c r="C171" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="D171" t="s">
         <v>433</v>
@@ -4459,7 +4459,7 @@
         <v>261</v>
       </c>
       <c r="C181" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="D181" t="s">
         <v>443</v>
@@ -4515,7 +4515,7 @@
         <v>261</v>
       </c>
       <c r="C185" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D185" t="s">
         <v>447</v>
@@ -4599,7 +4599,7 @@
         <v>259</v>
       </c>
       <c r="C191" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="D191" t="s">
         <v>453</v>
@@ -4683,7 +4683,7 @@
         <v>259</v>
       </c>
       <c r="C197" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D197" t="s">
         <v>459</v>
@@ -4823,7 +4823,7 @@
         <v>259</v>
       </c>
       <c r="C207" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="D207" t="s">
         <v>469</v>
@@ -4837,7 +4837,7 @@
         <v>261</v>
       </c>
       <c r="C208" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="D208" t="s">
         <v>470</v>
@@ -4851,7 +4851,7 @@
         <v>261</v>
       </c>
       <c r="C209" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="D209" t="s">
         <v>471</v>
@@ -4865,7 +4865,7 @@
         <v>261</v>
       </c>
       <c r="C210" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="D210" t="s">
         <v>472</v>
@@ -4879,7 +4879,7 @@
         <v>261</v>
       </c>
       <c r="C211" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="D211" t="s">
         <v>473</v>
@@ -4893,7 +4893,7 @@
         <v>261</v>
       </c>
       <c r="C212" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D212" t="s">
         <v>474</v>
@@ -5117,7 +5117,7 @@
         <v>261</v>
       </c>
       <c r="C228" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D228" t="s">
         <v>490</v>
@@ -5159,7 +5159,7 @@
         <v>261</v>
       </c>
       <c r="C231" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D231" t="s">
         <v>493</v>
@@ -5201,7 +5201,7 @@
         <v>259</v>
       </c>
       <c r="C234" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="D234" t="s">
         <v>496</v>
@@ -5271,7 +5271,7 @@
         <v>259</v>
       </c>
       <c r="C239" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="D239" t="s">
         <v>501</v>
@@ -5369,7 +5369,7 @@
         <v>261</v>
       </c>
       <c r="C246" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D246" t="s">
         <v>508</v>
@@ -5397,7 +5397,7 @@
         <v>261</v>
       </c>
       <c r="C248" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D248" t="s">
         <v>510</v>
@@ -5411,7 +5411,7 @@
         <v>261</v>
       </c>
       <c r="C249" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="D249" t="s">
         <v>511</v>

</xml_diff>